<commit_message>
added excel download button, and dynamic co2e calculation
</commit_message>
<xml_diff>
--- a/data/animals.xlsx
+++ b/data/animals.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25FCF5A1-9F03-4D01-8C49-E6E694948999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mim26609\PycharmProjects\OptiGOBTimeSeries\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B8E3B6-F2D5-4662-94B5-AD723B36C161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cattle" sheetId="1" r:id="rId1"/>
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="57">
   <si>
     <t>Abatement</t>
   </si>
@@ -78,21 +83,9 @@
     <t>unit</t>
   </si>
   <si>
-    <t>CH4</t>
-  </si>
-  <si>
     <t>kt</t>
   </si>
   <si>
-    <t>N2O</t>
-  </si>
-  <si>
-    <t>CO2</t>
-  </si>
-  <si>
-    <t>CO2e</t>
-  </si>
-  <si>
     <t>area_dairy</t>
   </si>
   <si>
@@ -202,6 +195,21 @@
   </si>
   <si>
     <t>hnv_area_ratio</t>
+  </si>
+  <si>
+    <t>ch4</t>
+  </si>
+  <si>
+    <t>n2o</t>
+  </si>
+  <si>
+    <t>co2e</t>
+  </si>
+  <si>
+    <t>co2</t>
+  </si>
+  <si>
+    <t>nh3</t>
   </si>
 </sst>
 </file>
@@ -601,23 +609,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.4140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.83203125" customWidth="1"/>
     <col min="6" max="7" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="14.58203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="14.58203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="18" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="14.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21">
@@ -878,10 +886,10 @@
     </row>
     <row r="6" spans="1:21">
       <c r="A6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C6" s="1">
         <v>2.1</v>
@@ -943,10 +951,10 @@
     </row>
     <row r="7" spans="1:21">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1">
         <v>0.1</v>
@@ -1008,10 +1016,10 @@
     </row>
     <row r="8" spans="1:21">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="1">
         <v>0.3</v>
@@ -1073,10 +1081,10 @@
     </row>
     <row r="9" spans="1:21">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1">
         <v>73.900000000000006</v>
@@ -1138,10 +1146,10 @@
     </row>
     <row r="10" spans="1:21">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2">
         <v>6255.4</v>
@@ -1203,10 +1211,10 @@
     </row>
     <row r="11" spans="1:21">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2">
         <v>4170.2</v>
@@ -1268,10 +1276,10 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C12" s="3">
         <v>54202500</v>
@@ -1333,10 +1341,10 @@
     </row>
     <row r="13" spans="1:21">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C13" s="3">
         <v>2421607</v>
@@ -1398,10 +1406,10 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C14" s="3">
         <v>56624107</v>
@@ -1463,10 +1471,10 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C15" s="3">
         <v>27439</v>
@@ -1528,10 +1536,10 @@
     </row>
     <row r="16" spans="1:21">
       <c r="A16" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C16" s="2">
         <v>1390.1</v>
@@ -1593,10 +1601,10 @@
     </row>
     <row r="17" spans="1:21">
       <c r="A17" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C17" s="3">
         <v>13895</v>
@@ -1658,10 +1666,10 @@
     </row>
     <row r="18" spans="1:21">
       <c r="A18" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C18" s="1">
         <v>966</v>
@@ -1723,10 +1731,10 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C19" s="1">
         <v>111</v>
@@ -1788,10 +1796,10 @@
     </row>
     <row r="20" spans="1:21">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C20" s="1">
         <v>362</v>
@@ -1853,10 +1861,10 @@
     </row>
     <row r="21" spans="1:21">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C21" s="1">
         <v>0.37</v>
@@ -1918,10 +1926,10 @@
     </row>
     <row r="22" spans="1:21">
       <c r="A22" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C22" s="1">
         <v>0.39</v>
@@ -1983,10 +1991,10 @@
     </row>
     <row r="23" spans="1:21">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C23" s="1">
         <v>0.02</v>
@@ -2048,10 +2056,10 @@
     </row>
     <row r="24" spans="1:21">
       <c r="A24" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C24" s="3">
         <v>5918</v>
@@ -2119,17 +2127,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{068914BF-AE90-4BE8-894C-61EC99CA55D7}">
   <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.58203125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.58203125" bestFit="1" customWidth="1"/>
     <col min="9" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.58203125" bestFit="1" customWidth="1"/>
     <col min="13" max="15" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2228,43 +2236,43 @@
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="H3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="L3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -2274,10 +2282,10 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C5" s="1">
         <v>15</v>
@@ -2321,10 +2329,10 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1">
         <v>0.2</v>
@@ -2368,10 +2376,10 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1">
         <v>0</v>
@@ -2415,10 +2423,10 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="1">
         <v>476.2</v>
@@ -2460,12 +2468,12 @@
         <v>554.70000000000005</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" ht="14.5">
       <c r="A9" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -2509,10 +2517,10 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10" s="2">
         <v>55453.7</v>
@@ -2556,10 +2564,10 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C11" s="2">
         <v>55453.7</v>
@@ -2603,10 +2611,10 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
@@ -2650,10 +2658,10 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2">
         <v>1322672.5</v>
@@ -2697,10 +2705,10 @@
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C14" s="1">
         <v>0</v>
@@ -2744,10 +2752,10 @@
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C15" s="1">
         <v>0</v>
@@ -2791,10 +2799,10 @@
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C16" s="1">
         <v>0</v>
@@ -2838,10 +2846,10 @@
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="1" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C17" s="1">
         <v>1.1000000000000001</v>
@@ -2885,10 +2893,10 @@
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" s="1">
         <v>1.3</v>
@@ -2932,10 +2940,10 @@
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="1">
         <v>0.1</v>
@@ -2979,10 +2987,10 @@
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C20" s="2">
         <v>205096.1</v>
@@ -3032,11 +3040,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D80CC04-5781-4AB2-AD88-17D811E13974}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>10</v>
@@ -3045,16 +3053,16 @@
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3203,63 +3211,63 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12AE4ACF-1B07-432B-B403-AB02D8214878}">
   <dimension ref="A1:V18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="9" width="21.28515625" customWidth="1"/>
+    <col min="1" max="1" width="15.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="9" width="21.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" t="s">
-        <v>49</v>
-      </c>
       <c r="I1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="S1" s="4"/>
     </row>
     <row r="2" spans="1:22">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -3269,10 +3277,10 @@
     </row>
     <row r="4" spans="1:22">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C4" s="5">
         <v>7.1881986300011903E-5</v>
@@ -3304,10 +3312,10 @@
     </row>
     <row r="5" spans="1:22">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -3339,10 +3347,10 @@
     </row>
     <row r="6" spans="1:22">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C6" s="5">
         <v>1.1401233025364475E-3</v>
@@ -3374,10 +3382,10 @@
     </row>
     <row r="7" spans="1:22">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C7" s="5">
         <v>3.1528189189367808E-3</v>
@@ -3409,10 +3417,10 @@
     </row>
     <row r="8" spans="1:22">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -3444,10 +3452,10 @@
     </row>
     <row r="9" spans="1:22">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C9" s="8">
         <v>141000</v>

</xml_diff>

<commit_message>
fixed database issue, added first optimisation iteration
</commit_message>
<xml_diff>
--- a/data/animals.xlsx
+++ b/data/animals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mim26609\PycharmProjects\OptiGOBTimeSeries\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B8E3B6-F2D5-4662-94B5-AD723B36C161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB311FE2-CAFE-4C9C-981C-C54C58301A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cattle" sheetId="1" r:id="rId1"/>
@@ -221,7 +221,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0E+00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,26 +609,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U24"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.4140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.83203125" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
     <col min="6" max="7" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -690,7 +690,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -753,7 +753,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -816,7 +816,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -864,7 +864,7 @@
         <v>10</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R4" s="1" t="s">
         <v>10</v>
@@ -879,12 +879,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
@@ -949,7 +949,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>53</v>
       </c>
@@ -1014,7 +1014,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>55</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>1.47</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>54</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>46.51</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>9980</v>
       </c>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -1404,7 +1404,7 @@
         <v>3008317</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>3008317</v>
       </c>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>26203</v>
       </c>
     </row>
-    <row r="16" spans="1:21">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>3326.7</v>
       </c>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>6228</v>
       </c>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="21" spans="1:21">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="24" spans="1:21">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>32</v>
       </c>
@@ -2127,21 +2127,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{068914BF-AE90-4BE8-894C-61EC99CA55D7}">
   <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.4140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.58203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.58203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.58203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="15" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2230,7 +2230,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -2275,12 +2275,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>52</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>12.4</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>53</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>55</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>87.9</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>54</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>554.70000000000005</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="14.5">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>595647.1</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>6891.5</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>6891.5</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>198549</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>299336.40000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>55121.9</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -2797,7 +2797,7 @@
         <v>6348.2</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>20662.099999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>56</v>
       </c>
@@ -2891,7 +2891,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -2938,7 +2938,7 @@
         <v>18.3</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -3040,9 +3040,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D80CC04-5781-4AB2-AD88-17D811E13974}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>2020</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2021</v>
       </c>
@@ -3111,7 +3111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2022</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2023</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2024</v>
       </c>
@@ -3180,7 +3180,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2025</v>
       </c>
@@ -3211,13 +3211,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12AE4ACF-1B07-432B-B403-AB02D8214878}">
   <dimension ref="A1:V18"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.4140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="9" width="21.25" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="9" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="S1" s="4"/>
     </row>
-    <row r="2" spans="1:22">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -3270,12 +3270,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:22">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -3310,7 +3310,7 @@
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
     </row>
-    <row r="5" spans="1:22">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -3345,7 +3345,7 @@
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>55</v>
       </c>
@@ -3380,7 +3380,7 @@
       <c r="U6" s="6"/>
       <c r="V6" s="6"/>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -3415,7 +3415,7 @@
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -3450,7 +3450,7 @@
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:22">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -3485,7 +3485,7 @@
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
       <c r="D10" s="7"/>
       <c r="F10" s="7"/>
@@ -3498,15 +3498,15 @@
       <c r="M10" s="7"/>
       <c r="N10" s="4"/>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
       <c r="N11" s="4"/>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -3521,27 +3521,27 @@
       <c r="M13" s="4"/>
       <c r="N13" s="9"/>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B14" s="4"/>
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
     </row>
-    <row r="15" spans="1:22">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="4:4">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D17" s="8"/>
     </row>
-    <row r="18" spans="4:4">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D18" s="8"/>
     </row>
   </sheetData>

</xml_diff>